<commit_message>
* refactored `map_etf_asset_class.py` and `WFA_to_positions.py` to be more object oriented and have more consistent coding style
</commit_message>
<xml_diff>
--- a/Morningstar_Asset_Stats/morningstar_stats.xlsx
+++ b/Morningstar_Asset_Stats/morningstar_stats.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11208"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10525"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bfraenkel/Documents/Code/Fin_Think/Morningstar_Asset_Correlation/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bfraenkel/Documents/Code/Financial_Plan/Morningstar_Asset_Stats/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{555CA7F6-D1F6-E945-BBE2-42610A50C59F}" xr6:coauthVersionLast="40" xr6:coauthVersionMax="40" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B7E2A5D-895A-A645-ABF5-668710798CC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="460" windowWidth="38400" windowHeight="21140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Stats" sheetId="1" r:id="rId1"/>
@@ -682,6 +682,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:O15"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="17.1640625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A1" t="s">

</xml_diff>